<commit_message>
Pass on REACH data nodification.
</commit_message>
<xml_diff>
--- a/inst/extdata/emissions/REACH_copper_prtd.xlsx
+++ b/inst/extdata/emissions/REACH_copper_prtd.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://miljodir-my.sharepoint.com/personal/espen_wigaard_miljodir_no/Documents/Vedlegg/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAW\Local Documents\EXPECT AEP\EXPECT_AEP_R_Project\inst\extdata\emissions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{0370FB41-9541-4325-94C1-59A7EE622D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0F063BA-0839-4BB3-9781-4136002251A7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FB5AA9-987E-40F7-B125-5BF861E4AEFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35115" yWindow="435" windowWidth="21300" windowHeight="15330" activeTab="1" xr2:uid="{4DA265A8-543D-459F-B447-B2F48819DC54}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{4DA265A8-543D-459F-B447-B2F48819DC54}"/>
   </bookViews>
   <sheets>
     <sheet name="Forklaring" sheetId="5" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="201">
   <si>
     <t>AmountYear</t>
   </si>
@@ -66,84 +66,39 @@
     <t>Beskrivelse</t>
   </si>
   <si>
-    <t>86.8336585179</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>0.000021988769999999996</t>
-  </si>
-  <si>
     <t>Annen tjenesteyting</t>
   </si>
   <si>
-    <t>820.5267</t>
-  </si>
-  <si>
     <t>Bergverksdrift og utvinning</t>
   </si>
   <si>
-    <t>1.2853754968000002</t>
-  </si>
-  <si>
     <t>Bygge- og anleggsvirksomhet</t>
   </si>
   <si>
-    <t>53024.96756487536</t>
-  </si>
-  <si>
     <t>Industri</t>
   </si>
   <si>
-    <t>1833.5758884962493</t>
-  </si>
-  <si>
     <t>Jordbruk, skogbruk og fiske</t>
   </si>
   <si>
-    <t>0.0139324115</t>
-  </si>
-  <si>
     <t>Kulturell virksomhet, underholdning og fritidsaktiviteter</t>
   </si>
   <si>
-    <t>0.0019375</t>
-  </si>
-  <si>
     <t>Omsetning og drift av fast eiendom</t>
   </si>
   <si>
-    <t>0.812001291873435</t>
-  </si>
-  <si>
     <t>Transport og lagring</t>
   </si>
   <si>
-    <t>0.07395199999999999</t>
-  </si>
-  <si>
     <t>Vannforsyning, avløps- og renovasjonsvirksomhet</t>
   </si>
   <si>
-    <t>12.090757980102667</t>
-  </si>
-  <si>
     <t>Varehandel, reparasjon av motorvogner</t>
   </si>
   <si>
-    <t>42.687122408408285</t>
-  </si>
-  <si>
-    <t>0.000001328</t>
-  </si>
-  <si>
-    <t>561.7192634</t>
-  </si>
-  <si>
-    <t>0.9770535927799989</t>
-  </si>
-  <si>
     <t>0.0000512</t>
   </si>
   <si>
@@ -156,138 +111,33 @@
     <t>Forretningsmessig tjenesteyting</t>
   </si>
   <si>
-    <t>56397.83415313219</t>
-  </si>
-  <si>
-    <t>1911.5584339999978</t>
-  </si>
-  <si>
-    <t>0.0117045215</t>
-  </si>
-  <si>
-    <t>0.00126</t>
-  </si>
-  <si>
-    <t>1.62399999999999</t>
-  </si>
-  <si>
-    <t>0.7182324659754898</t>
-  </si>
-  <si>
-    <t>4063.929616881107</t>
-  </si>
-  <si>
-    <t>817.088842</t>
-  </si>
-  <si>
-    <t>1.9421949579539985</t>
-  </si>
-  <si>
-    <t>7.41599999999999e-8</t>
-  </si>
-  <si>
     <t>Elektrisitets-, gass-, damp- og varmtvannsforsyning</t>
   </si>
   <si>
-    <t>58366.78017287691</t>
-  </si>
-  <si>
-    <t>1746.867406354999</t>
-  </si>
-  <si>
-    <t>0.0174549503292</t>
-  </si>
-  <si>
-    <t>0.002417499999999999</t>
-  </si>
-  <si>
-    <t>0.5800013348799999</t>
-  </si>
-  <si>
-    <t>0.1479039999999999</t>
-  </si>
-  <si>
-    <t>16.327402294250895</t>
-  </si>
-  <si>
-    <t>58.28346077204123</t>
-  </si>
-  <si>
     <t>550.7568</t>
   </si>
   <si>
-    <t>12.5073645270394</t>
-  </si>
-  <si>
     <t>0.0000612</t>
   </si>
   <si>
-    <t>58547.522422945345</t>
-  </si>
-  <si>
-    <t>1238.5270110000001</t>
-  </si>
-  <si>
-    <t>0.032014759409999996</t>
-  </si>
-  <si>
-    <t>0.00402</t>
-  </si>
-  <si>
     <t>0.232000000000003</t>
   </si>
   <si>
-    <t>13.969691591322588</t>
-  </si>
-  <si>
-    <t>60.42287644245364</t>
-  </si>
-  <si>
     <t>744.412115</t>
   </si>
   <si>
-    <t>1.11616699513586</t>
-  </si>
-  <si>
-    <t>6949.458314472632</t>
-  </si>
-  <si>
-    <t>499.17731899999995</t>
-  </si>
-  <si>
     <t>0.003</t>
   </si>
   <si>
     <t>0.58</t>
   </si>
   <si>
-    <t>3.83148195893011</t>
-  </si>
-  <si>
-    <t>-62.166816462951985</t>
-  </si>
-  <si>
     <t>599.1080000000001</t>
   </si>
   <si>
-    <t>0.8938951997139201</t>
-  </si>
-  <si>
-    <t>10434.835462404693</t>
-  </si>
-  <si>
-    <t>-545.383885</t>
-  </si>
-  <si>
-    <t>0.0057</t>
-  </si>
-  <si>
     <t>0.463999999999998</t>
   </si>
   <si>
-    <t>0.8348878412695961</t>
-  </si>
-  <si>
     <t>Netto Mengde (tonn)</t>
   </si>
   <si>
@@ -366,124 +216,64 @@
     <t>Tekst</t>
   </si>
   <si>
-    <t>0.811999999999995</t>
-  </si>
-  <si>
     <t xml:space="preserve"> BRENSELTILSETNINGER</t>
   </si>
   <si>
-    <t>716.0267</t>
-  </si>
-  <si>
     <t>Absorpsjons/ og adsorpsjonsmaterialer</t>
   </si>
   <si>
-    <t>0.23761759999999996</t>
-  </si>
-  <si>
     <t>ANDRE SMØREMIDLER</t>
   </si>
   <si>
-    <t>0.00000160896</t>
-  </si>
-  <si>
     <t>ARMERINGSMIDLER</t>
   </si>
   <si>
-    <t>1.3502159999999999</t>
-  </si>
-  <si>
     <t>Bindemidler</t>
   </si>
   <si>
-    <t>2460.47245096512</t>
-  </si>
-  <si>
     <t>Biocider</t>
   </si>
   <si>
-    <t>104.5</t>
-  </si>
-  <si>
     <t>Borekjemikalier inkl råolje/gass</t>
   </si>
   <si>
-    <t>0.00527</t>
-  </si>
-  <si>
     <t>BOREOLJER</t>
   </si>
   <si>
-    <t>0.27702</t>
-  </si>
-  <si>
     <t>BUNNFELLINGSHINDRENDE MIDLER, GENERELT</t>
   </si>
   <si>
-    <t>0.011650853446</t>
-  </si>
-  <si>
     <t>Fyllingsmidler</t>
   </si>
   <si>
-    <t>0.6897628999999998</t>
-  </si>
-  <si>
     <t>GJØDNING, GENERELT</t>
   </si>
   <si>
-    <t>11.084</t>
-  </si>
-  <si>
     <t>Impregnering</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>INSEKTSMIDDEL, INSEKTMIDLER OG ANDRE MIDLER MOT SKADEDYR PÅ PLANTER</t>
   </si>
   <si>
-    <t>2.5608630450000005</t>
-  </si>
-  <si>
     <t>Konstruksjonsmaterialer</t>
   </si>
   <si>
-    <t>0.0000017368</t>
-  </si>
-  <si>
     <t>Lim</t>
   </si>
   <si>
-    <t>1.7117688</t>
-  </si>
-  <si>
     <t>Maling</t>
   </si>
   <si>
     <t>PH-REGULERENDE MIDLER, GENERELT</t>
   </si>
   <si>
-    <t>134.98239999999998</t>
-  </si>
-  <si>
     <t>Prosessregulerendemidler</t>
   </si>
   <si>
-    <t>50.5</t>
-  </si>
-  <si>
     <t>Rengjøring</t>
   </si>
   <si>
-    <t>0.054</t>
-  </si>
-  <si>
     <t>Rustbeskyttelse</t>
-  </si>
-  <si>
-    <t>0.052</t>
   </si>
   <si>
     <t>SALT TIL GALVANISKE BAD</t>
@@ -912,22 +702,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1067,8 +858,8 @@
   <autoFilter ref="A1:C62" xr:uid="{BCD99A77-6934-4E99-8C1B-54ABCC140FC1}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D080CC97-425D-4B46-A4E2-B1B8FC4ED62B}" uniqueName="1" name="AmountYear" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{8BB0EFBC-97DF-46CA-83EA-A205B241C52A}" uniqueName="2" name="Netto Mengde (tonn)" queryTableFieldId="2" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{1525CC88-ADBE-4E58-8086-2F26CB88023A}" uniqueName="3" name="Beskrivelse" queryTableFieldId="3" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{8BB0EFBC-97DF-46CA-83EA-A205B241C52A}" uniqueName="2" name="Netto Mengde (tonn)" queryTableFieldId="2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1525CC88-ADBE-4E58-8086-2F26CB88023A}" uniqueName="3" name="Beskrivelse" queryTableFieldId="3" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1079,15 +870,15 @@
   <autoFilter ref="A1:C142" xr:uid="{CCDA5120-8910-49CF-ACD3-A8DEBF69B715}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7843A04F-20F8-4390-A62B-E988A1C91BAF}" uniqueName="1" name="AmountYear" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{3176676A-B9BF-41F1-A84D-C925960862FB}" uniqueName="2" name="Netto mengde i tonn" queryTableFieldId="2" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{FA89C65B-FAB6-4333-8C88-9D68053616B1}" uniqueName="3" name="Tekst" queryTableFieldId="3" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{3176676A-B9BF-41F1-A84D-C925960862FB}" uniqueName="2" name="Netto mengde i tonn" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{FA89C65B-FAB6-4333-8C88-9D68053616B1}" uniqueName="3" name="Tekst" queryTableFieldId="3" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1404,122 +1195,122 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8010FE5F-5D8C-4C1D-8019-14D83F682986}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>88</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1530,102 +1321,102 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4437D70C-BAF5-4080-8000-8BE92E6E5B78}">
   <dimension ref="A29:B40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>88</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1637,693 +1428,693 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79374472-9405-4124-A0D2-6C9DDEA4F4AC}">
   <dimension ref="A1:C62"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>76</v>
+      <c r="B1" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2018</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2">
+        <v>86.833658517900005</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
-      <c r="B3" t="s">
-        <v>4</v>
+      <c r="B3" s="2">
+        <v>2.1988769999999902E-5</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2018</v>
       </c>
-      <c r="B4" t="s">
-        <v>6</v>
+      <c r="B4" s="2">
+        <v>820.52670000000001</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2018</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
+      <c r="B5" s="2">
+        <v>1.2853754968</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2018</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
+      <c r="B6" s="2">
+        <v>53024.967564875296</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
+      <c r="B7" s="2">
+        <v>1833.5758884962399</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2018</v>
       </c>
-      <c r="B8" t="s">
-        <v>14</v>
+      <c r="B8" s="2">
+        <v>1.39324115E-2</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2018</v>
       </c>
-      <c r="B9" t="s">
-        <v>16</v>
+      <c r="B9" s="2">
+        <v>1.9375E-3</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
-      <c r="B10" t="s">
-        <v>18</v>
+      <c r="B10" s="2">
+        <v>0.81200129187343495</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2018</v>
       </c>
-      <c r="B11" t="s">
-        <v>20</v>
+      <c r="B11" s="2">
+        <v>7.3951999999999907E-2</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2018</v>
       </c>
-      <c r="B12" t="s">
-        <v>22</v>
+      <c r="B12" s="2">
+        <v>12.0907579801026</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2019</v>
       </c>
-      <c r="B13" t="s">
-        <v>24</v>
+      <c r="B13" s="2">
+        <v>42.6871224084082</v>
       </c>
       <c r="C13" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2019</v>
       </c>
-      <c r="B14" t="s">
-        <v>25</v>
+      <c r="B14" s="2">
+        <v>1.328E-6</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2019</v>
       </c>
-      <c r="B15" t="s">
-        <v>26</v>
+      <c r="B15" s="2">
+        <v>561.71926340000005</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2019</v>
       </c>
-      <c r="B16" t="s">
-        <v>27</v>
+      <c r="B16" s="2">
+        <v>0.97705359277999804</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2019</v>
       </c>
-      <c r="B17" t="s">
-        <v>28</v>
+      <c r="B17" s="2">
+        <v>5.1199999999999998E-5</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2019</v>
       </c>
-      <c r="B18" t="s">
-        <v>30</v>
+      <c r="B18" s="2">
+        <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2019</v>
       </c>
-      <c r="B19" t="s">
-        <v>32</v>
+      <c r="B19" s="2">
+        <v>56397.834153132098</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2019</v>
       </c>
-      <c r="B20" t="s">
-        <v>33</v>
+      <c r="B20" s="2">
+        <v>1911.55843399999</v>
       </c>
       <c r="C20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2019</v>
       </c>
-      <c r="B21" t="s">
-        <v>34</v>
+      <c r="B21" s="2">
+        <v>1.17045215E-2</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2019</v>
       </c>
-      <c r="B22" t="s">
-        <v>35</v>
+      <c r="B22" s="2">
+        <v>1.2600000000000001E-3</v>
       </c>
       <c r="C22" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2019</v>
       </c>
-      <c r="B23" t="s">
-        <v>36</v>
+      <c r="B23" s="2">
+        <v>1.6239999999999899</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2019</v>
       </c>
-      <c r="B24" t="s">
-        <v>37</v>
+      <c r="B24" s="2">
+        <v>0.71823246597548895</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2020</v>
       </c>
-      <c r="B25" t="s">
-        <v>38</v>
+      <c r="B25" s="2">
+        <v>4063.9296168811002</v>
       </c>
       <c r="C25" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2020</v>
       </c>
-      <c r="B26" t="s">
-        <v>39</v>
+      <c r="B26" s="2">
+        <v>817.088842</v>
       </c>
       <c r="C26" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2020</v>
       </c>
-      <c r="B27" t="s">
-        <v>40</v>
+      <c r="B27" s="2">
+        <v>1.9421949579539901</v>
       </c>
       <c r="C27" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2020</v>
       </c>
-      <c r="B28" t="s">
-        <v>41</v>
+      <c r="B28" s="2">
+        <v>7.4159999999999904E-8</v>
       </c>
       <c r="C28" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2020</v>
       </c>
-      <c r="B29" t="s">
-        <v>43</v>
+      <c r="B29" s="2">
+        <v>58366.780172876897</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2020</v>
       </c>
-      <c r="B30" t="s">
-        <v>44</v>
+      <c r="B30" s="2">
+        <v>1746.86740635499</v>
       </c>
       <c r="C30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2020</v>
       </c>
-      <c r="B31" t="s">
-        <v>45</v>
+      <c r="B31" s="2">
+        <v>1.7454950329200001E-2</v>
       </c>
       <c r="C31" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2020</v>
       </c>
-      <c r="B32" t="s">
-        <v>46</v>
+      <c r="B32" s="2">
+        <v>2.41749999999999E-3</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2020</v>
       </c>
-      <c r="B33" t="s">
-        <v>47</v>
+      <c r="B33" s="2">
+        <v>0.58000133487999905</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2020</v>
       </c>
-      <c r="B34" t="s">
-        <v>48</v>
+      <c r="B34" s="2">
+        <v>0.14790399999999901</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2020</v>
       </c>
-      <c r="B35" t="s">
-        <v>49</v>
+      <c r="B35" s="2">
+        <v>16.327402294250799</v>
       </c>
       <c r="C35" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2021</v>
       </c>
-      <c r="B36" t="s">
-        <v>50</v>
+      <c r="B36" s="2">
+        <v>58.283460772041202</v>
       </c>
       <c r="C36" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2021</v>
       </c>
-      <c r="B37" t="s">
-        <v>51</v>
+      <c r="B37" s="2">
+        <v>550.7568</v>
       </c>
       <c r="C37" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2021</v>
       </c>
-      <c r="B38" t="s">
-        <v>52</v>
+      <c r="B38" s="2">
+        <v>12.5073645270394</v>
       </c>
       <c r="C38" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2021</v>
       </c>
-      <c r="B39" t="s">
-        <v>53</v>
+      <c r="B39" s="2">
+        <v>6.1199999999999997E-5</v>
       </c>
       <c r="C39" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2021</v>
       </c>
-      <c r="B40" t="s">
-        <v>54</v>
+      <c r="B40" s="2">
+        <v>58547.522422945302</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2021</v>
       </c>
-      <c r="B41" t="s">
-        <v>55</v>
+      <c r="B41" s="2">
+        <v>1238.5270109999999</v>
       </c>
       <c r="C41" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2021</v>
       </c>
-      <c r="B42" t="s">
-        <v>56</v>
+      <c r="B42" s="2">
+        <v>3.2014759409999899E-2</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2021</v>
       </c>
-      <c r="B43" t="s">
-        <v>57</v>
+      <c r="B43" s="2">
+        <v>4.0200000000000001E-3</v>
       </c>
       <c r="C43" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2021</v>
       </c>
-      <c r="B44" t="s">
-        <v>58</v>
+      <c r="B44" s="2">
+        <v>0.23200000000000301</v>
       </c>
       <c r="C44" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2021</v>
       </c>
-      <c r="B45" t="s">
-        <v>20</v>
+      <c r="B45" s="2">
+        <v>7.3951999999999907E-2</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2021</v>
       </c>
-      <c r="B46" t="s">
-        <v>59</v>
+      <c r="B46" s="2">
+        <v>13.969691591322499</v>
       </c>
       <c r="C46" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2022</v>
       </c>
-      <c r="B47" t="s">
-        <v>60</v>
+      <c r="B47" s="2">
+        <v>60.4228764424536</v>
       </c>
       <c r="C47" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2022</v>
       </c>
-      <c r="B48" t="s">
-        <v>61</v>
+      <c r="B48" s="2">
+        <v>744.41211499999997</v>
       </c>
       <c r="C48" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2022</v>
       </c>
-      <c r="B49" t="s">
-        <v>62</v>
+      <c r="B49" s="2">
+        <v>1.1161669951358599</v>
       </c>
       <c r="C49" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2022</v>
       </c>
-      <c r="B50" t="s">
-        <v>63</v>
+      <c r="B50" s="2">
+        <v>6949.4583144726303</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2022</v>
       </c>
-      <c r="B51" t="s">
-        <v>64</v>
+      <c r="B51" s="2">
+        <v>499.17731899999899</v>
       </c>
       <c r="C51" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2022</v>
       </c>
-      <c r="B52" t="s">
-        <v>65</v>
+      <c r="B52" s="2">
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C52" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2022</v>
       </c>
-      <c r="B53" t="s">
-        <v>66</v>
+      <c r="B53" s="2">
+        <v>0.57999999999999996</v>
       </c>
       <c r="C53" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2022</v>
       </c>
-      <c r="B54" t="s">
-        <v>67</v>
+      <c r="B54" s="2">
+        <v>3.8314819589301101</v>
       </c>
       <c r="C54" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2023</v>
       </c>
-      <c r="B55" t="s">
-        <v>68</v>
+      <c r="B55" s="2">
+        <v>-62.1668164629519</v>
       </c>
       <c r="C55" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2023</v>
       </c>
-      <c r="B56" t="s">
-        <v>69</v>
+      <c r="B56" s="2">
+        <v>599.10799999999995</v>
       </c>
       <c r="C56" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2023</v>
       </c>
-      <c r="B57" t="s">
-        <v>70</v>
+      <c r="B57" s="2">
+        <v>0.89389519971391995</v>
       </c>
       <c r="C57" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2023</v>
       </c>
-      <c r="B58" t="s">
-        <v>71</v>
+      <c r="B58" s="2">
+        <v>10434.835462404601</v>
       </c>
       <c r="C58" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2023</v>
       </c>
-      <c r="B59" t="s">
-        <v>72</v>
+      <c r="B59" s="2">
+        <v>-545.38388499999996</v>
       </c>
       <c r="C59" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2023</v>
       </c>
-      <c r="B60" t="s">
-        <v>73</v>
+      <c r="B60" s="2">
+        <v>5.7000000000000002E-3</v>
       </c>
       <c r="C60" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2023</v>
       </c>
-      <c r="B61" t="s">
-        <v>74</v>
+      <c r="B61" s="2">
+        <v>0.46399999999999803</v>
       </c>
       <c r="C61" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2023</v>
       </c>
-      <c r="B62" t="s">
-        <v>75</v>
+      <c r="B62" s="2">
+        <v>0.83488784126959603</v>
       </c>
       <c r="C62" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2337,1573 +2128,1573 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BF79F73-0A3E-4188-9F8B-21D3192D1371}">
   <dimension ref="A1:C142"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>266</v>
+      <c r="B1" s="2" t="s">
+        <v>196</v>
       </c>
       <c r="C1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2018</v>
       </c>
-      <c r="B2" t="s">
-        <v>102</v>
+      <c r="B2" s="2">
+        <v>0.81199999999999495</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
-      <c r="B3" t="s">
-        <v>104</v>
+      <c r="B3" s="2">
+        <v>716.02670000000001</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2018</v>
       </c>
-      <c r="B4" t="s">
-        <v>106</v>
+      <c r="B4" s="2">
+        <v>0.23761759999999901</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2018</v>
       </c>
-      <c r="B5" t="s">
-        <v>108</v>
+      <c r="B5" s="2">
+        <v>1.6089599999999999E-6</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2018</v>
       </c>
-      <c r="B6" t="s">
-        <v>110</v>
+      <c r="B6" s="2">
+        <v>1.3502159999999901</v>
       </c>
       <c r="C6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
-      <c r="B7" t="s">
-        <v>112</v>
+      <c r="B7" s="2">
+        <v>2460.4724509651201</v>
       </c>
       <c r="C7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2018</v>
       </c>
-      <c r="B8" t="s">
-        <v>114</v>
+      <c r="B8" s="2">
+        <v>104.5</v>
       </c>
       <c r="C8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2018</v>
       </c>
-      <c r="B9" t="s">
-        <v>116</v>
+      <c r="B9" s="2">
+        <v>5.2700000000000004E-3</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
-      <c r="B10" t="s">
-        <v>118</v>
+      <c r="B10" s="2">
+        <v>0.27701999999999999</v>
       </c>
       <c r="C10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2018</v>
       </c>
-      <c r="B11" t="s">
-        <v>120</v>
+      <c r="B11" s="2">
+        <v>1.1650853446E-2</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2018</v>
       </c>
-      <c r="B12" t="s">
-        <v>122</v>
+      <c r="B12" s="2">
+        <v>0.68976289999999896</v>
       </c>
       <c r="C12" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2018</v>
       </c>
-      <c r="B13" t="s">
-        <v>124</v>
+      <c r="B13" s="2">
+        <v>11.084</v>
       </c>
       <c r="C13" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2018</v>
       </c>
-      <c r="B14" t="s">
-        <v>126</v>
+      <c r="B14" s="2">
+        <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2018</v>
       </c>
-      <c r="B15" t="s">
-        <v>128</v>
+      <c r="B15" s="2">
+        <v>2.5608630450000001</v>
       </c>
       <c r="C15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2018</v>
       </c>
-      <c r="B16" t="s">
-        <v>130</v>
+      <c r="B16" s="2">
+        <v>1.7368E-6</v>
       </c>
       <c r="C16" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2018</v>
       </c>
-      <c r="B17" t="s">
-        <v>132</v>
+      <c r="B17" s="2">
+        <v>1.7117688</v>
       </c>
       <c r="C17" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2018</v>
       </c>
-      <c r="B18" t="s">
-        <v>30</v>
+      <c r="B18" s="2">
+        <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2018</v>
       </c>
-      <c r="B19" t="s">
-        <v>135</v>
+      <c r="B19" s="2">
+        <v>134.98239999999899</v>
       </c>
       <c r="C19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2018</v>
       </c>
-      <c r="B20" t="s">
-        <v>137</v>
+      <c r="B20" s="2">
+        <v>50.5</v>
       </c>
       <c r="C20" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2018</v>
       </c>
-      <c r="B21" t="s">
-        <v>139</v>
+      <c r="B21" s="2">
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="C21" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2018</v>
       </c>
-      <c r="B22" t="s">
-        <v>141</v>
+      <c r="B22" s="2">
+        <v>5.1999999999999998E-2</v>
       </c>
       <c r="C22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2018</v>
       </c>
-      <c r="B23" t="s">
-        <v>143</v>
+      <c r="B23" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="C23" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2018</v>
       </c>
-      <c r="B24" t="s">
-        <v>145</v>
+      <c r="B24" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2018</v>
       </c>
-      <c r="B25" t="s">
-        <v>147</v>
+      <c r="B25" s="2" t="s">
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2018</v>
       </c>
-      <c r="B26" t="s">
-        <v>149</v>
+      <c r="B26" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="C26" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2019</v>
       </c>
-      <c r="B27" t="s">
-        <v>151</v>
+      <c r="B27" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2019</v>
       </c>
-      <c r="B28" t="s">
-        <v>152</v>
+      <c r="B28" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="C28" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2019</v>
       </c>
-      <c r="B29" t="s">
-        <v>153</v>
+      <c r="B29" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="C29" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2019</v>
       </c>
-      <c r="B30" t="s">
-        <v>154</v>
+      <c r="B30" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2019</v>
       </c>
-      <c r="B31" t="s">
-        <v>155</v>
+      <c r="B31" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="C31" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2019</v>
       </c>
-      <c r="B32" t="s">
-        <v>156</v>
+      <c r="B32" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2019</v>
       </c>
-      <c r="B33" t="s">
-        <v>28</v>
+      <c r="B33" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="C33" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2019</v>
       </c>
-      <c r="B34" t="s">
-        <v>158</v>
+      <c r="B34" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="C34" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2019</v>
       </c>
-      <c r="B35" t="s">
-        <v>65</v>
+      <c r="B35" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="C35" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2019</v>
       </c>
-      <c r="B36" t="s">
-        <v>160</v>
+      <c r="B36" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2019</v>
       </c>
-      <c r="B37" t="s">
-        <v>161</v>
+      <c r="B37" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2019</v>
       </c>
-      <c r="B38" t="s">
-        <v>162</v>
+      <c r="B38" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="C38" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2019</v>
       </c>
-      <c r="B39" t="s">
-        <v>164</v>
+      <c r="B39" s="2" t="s">
+        <v>94</v>
       </c>
       <c r="C39" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2019</v>
       </c>
-      <c r="B40" t="s">
-        <v>166</v>
+      <c r="B40" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="C40" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2019</v>
       </c>
-      <c r="B41" t="s">
-        <v>167</v>
+      <c r="B41" s="2" t="s">
+        <v>97</v>
       </c>
       <c r="C41" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2019</v>
       </c>
-      <c r="B42" t="s">
-        <v>168</v>
+      <c r="B42" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2019</v>
       </c>
-      <c r="B43" t="s">
-        <v>170</v>
+      <c r="B43" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="C43" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2019</v>
       </c>
-      <c r="B44" t="s">
-        <v>30</v>
+      <c r="B44" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C44" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2019</v>
       </c>
-      <c r="B45" t="s">
-        <v>171</v>
+      <c r="B45" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="C45" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2019</v>
       </c>
-      <c r="B46" t="s">
-        <v>172</v>
+      <c r="B46" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2019</v>
       </c>
-      <c r="B47" t="s">
-        <v>173</v>
+      <c r="B47" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="C47" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2019</v>
       </c>
-      <c r="B48" t="s">
-        <v>174</v>
+      <c r="B48" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2019</v>
       </c>
-      <c r="B49" t="s">
-        <v>175</v>
+      <c r="B49" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2019</v>
       </c>
-      <c r="B50" t="s">
-        <v>176</v>
+      <c r="B50" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="C50" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2019</v>
       </c>
-      <c r="B51" t="s">
-        <v>177</v>
+      <c r="B51" s="2" t="s">
+        <v>107</v>
       </c>
       <c r="C51" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2020</v>
       </c>
-      <c r="B52" t="s">
-        <v>66</v>
+      <c r="B52" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C52" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2020</v>
       </c>
-      <c r="B53" t="s">
-        <v>178</v>
+      <c r="B53" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="C53" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2020</v>
       </c>
-      <c r="B54" t="s">
-        <v>179</v>
+      <c r="B54" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="C54" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2020</v>
       </c>
-      <c r="B55" t="s">
-        <v>180</v>
+      <c r="B55" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="C55" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2020</v>
       </c>
-      <c r="B56" t="s">
-        <v>181</v>
+      <c r="B56" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="C56" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2020</v>
       </c>
-      <c r="B57" t="s">
-        <v>183</v>
+      <c r="B57" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="C57" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2020</v>
       </c>
-      <c r="B58" t="s">
-        <v>184</v>
+      <c r="B58" s="2" t="s">
+        <v>114</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2020</v>
       </c>
-      <c r="B59" t="s">
-        <v>185</v>
+      <c r="B59" s="2" t="s">
+        <v>115</v>
       </c>
       <c r="C59" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2020</v>
       </c>
-      <c r="B60" t="s">
-        <v>186</v>
+      <c r="B60" s="2" t="s">
+        <v>116</v>
       </c>
       <c r="C60" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2020</v>
       </c>
-      <c r="B61" t="s">
-        <v>187</v>
+      <c r="B61" s="2" t="s">
+        <v>117</v>
       </c>
       <c r="C61" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2020</v>
       </c>
-      <c r="B62" t="s">
-        <v>189</v>
+      <c r="B62" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="C62" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2020</v>
       </c>
-      <c r="B63" t="s">
-        <v>190</v>
+      <c r="B63" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="C63" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2020</v>
       </c>
-      <c r="B64" t="s">
-        <v>191</v>
+      <c r="B64" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="C64" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2020</v>
       </c>
-      <c r="B65" t="s">
-        <v>192</v>
+      <c r="B65" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="C65" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2020</v>
       </c>
-      <c r="B66" t="s">
-        <v>193</v>
+      <c r="B66" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="C66" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2020</v>
       </c>
-      <c r="B67" t="s">
-        <v>194</v>
+      <c r="B67" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="C67" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2020</v>
       </c>
-      <c r="B68" t="s">
-        <v>195</v>
+      <c r="B68" s="2" t="s">
+        <v>125</v>
       </c>
       <c r="C68" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2020</v>
       </c>
-      <c r="B69" t="s">
-        <v>196</v>
+      <c r="B69" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="C69" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2020</v>
       </c>
-      <c r="B70" t="s">
-        <v>197</v>
+      <c r="B70" s="2" t="s">
+        <v>127</v>
       </c>
       <c r="C70" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2020</v>
       </c>
-      <c r="B71" t="s">
-        <v>30</v>
+      <c r="B71" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C71" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2020</v>
       </c>
-      <c r="B72" t="s">
-        <v>198</v>
+      <c r="B72" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="C72" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2020</v>
       </c>
-      <c r="B73" t="s">
-        <v>200</v>
+      <c r="B73" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="C73" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2020</v>
       </c>
-      <c r="B74" t="s">
-        <v>201</v>
+      <c r="B74" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="C74" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2020</v>
       </c>
-      <c r="B75" t="s">
-        <v>202</v>
+      <c r="B75" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="C75" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2020</v>
       </c>
-      <c r="B76" t="s">
-        <v>203</v>
+      <c r="B76" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="C76" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2020</v>
       </c>
-      <c r="B77" t="s">
-        <v>204</v>
+      <c r="B77" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="C77" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2020</v>
       </c>
-      <c r="B78" t="s">
-        <v>205</v>
+      <c r="B78" s="2" t="s">
+        <v>135</v>
       </c>
       <c r="C78" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2021</v>
       </c>
-      <c r="B79" t="s">
-        <v>58</v>
+      <c r="B79" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="C79" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2021</v>
       </c>
-      <c r="B80" t="s">
-        <v>51</v>
+      <c r="B80" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C80" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2021</v>
       </c>
-      <c r="B81" t="s">
-        <v>206</v>
+      <c r="B81" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="C81" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2021</v>
       </c>
-      <c r="B82" t="s">
-        <v>207</v>
+      <c r="B82" s="2" t="s">
+        <v>137</v>
       </c>
       <c r="C82" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2021</v>
       </c>
-      <c r="B83" t="s">
-        <v>208</v>
+      <c r="B83" s="2" t="s">
+        <v>138</v>
       </c>
       <c r="C83" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2021</v>
       </c>
-      <c r="B84" t="s">
-        <v>209</v>
+      <c r="B84" s="2" t="s">
+        <v>139</v>
       </c>
       <c r="C84" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2021</v>
       </c>
-      <c r="B85" t="s">
-        <v>210</v>
+      <c r="B85" s="2" t="s">
+        <v>140</v>
       </c>
       <c r="C85" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2021</v>
       </c>
-      <c r="B86" t="s">
-        <v>53</v>
+      <c r="B86" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="C86" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2021</v>
       </c>
-      <c r="B87" t="s">
-        <v>211</v>
+      <c r="B87" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="C87" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2021</v>
       </c>
-      <c r="B88" t="s">
-        <v>212</v>
+      <c r="B88" s="2" t="s">
+        <v>142</v>
       </c>
       <c r="C88" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2021</v>
       </c>
-      <c r="B89" t="s">
-        <v>213</v>
+      <c r="B89" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="C89" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2021</v>
       </c>
-      <c r="B90" t="s">
-        <v>214</v>
+      <c r="B90" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="C90" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2021</v>
       </c>
-      <c r="B91" t="s">
-        <v>215</v>
+      <c r="B91" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="C91" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2021</v>
       </c>
-      <c r="B92" t="s">
-        <v>216</v>
+      <c r="B92" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="C92" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2021</v>
       </c>
-      <c r="B93" t="s">
-        <v>217</v>
+      <c r="B93" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="C93" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2021</v>
       </c>
-      <c r="B94" t="s">
-        <v>218</v>
+      <c r="B94" s="2" t="s">
+        <v>148</v>
       </c>
       <c r="C94" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2021</v>
       </c>
-      <c r="B95" t="s">
-        <v>219</v>
+      <c r="B95" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="C95" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2021</v>
       </c>
-      <c r="B96" t="s">
-        <v>220</v>
+      <c r="B96" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="C96" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2021</v>
       </c>
-      <c r="B97" t="s">
-        <v>222</v>
+      <c r="B97" s="2" t="s">
+        <v>152</v>
       </c>
       <c r="C97" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2021</v>
       </c>
-      <c r="B98" t="s">
-        <v>223</v>
+      <c r="B98" s="2" t="s">
+        <v>153</v>
       </c>
       <c r="C98" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2021</v>
       </c>
-      <c r="B99" t="s">
-        <v>224</v>
+      <c r="B99" s="2" t="s">
+        <v>154</v>
       </c>
       <c r="C99" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2021</v>
       </c>
-      <c r="B100" t="s">
-        <v>225</v>
+      <c r="B100" s="2" t="s">
+        <v>155</v>
       </c>
       <c r="C100" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2021</v>
       </c>
-      <c r="B101" t="s">
-        <v>226</v>
+      <c r="B101" s="2" t="s">
+        <v>156</v>
       </c>
       <c r="C101" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2022</v>
       </c>
-      <c r="B102" t="s">
-        <v>66</v>
+      <c r="B102" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C102" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2022</v>
       </c>
-      <c r="B103" t="s">
-        <v>61</v>
+      <c r="B103" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C103" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2022</v>
       </c>
-      <c r="B104" t="s">
-        <v>227</v>
+      <c r="B104" s="2" t="s">
+        <v>157</v>
       </c>
       <c r="C104" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2022</v>
       </c>
-      <c r="B105" t="s">
-        <v>228</v>
+      <c r="B105" s="2" t="s">
+        <v>158</v>
       </c>
       <c r="C105" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2022</v>
       </c>
-      <c r="B106" t="s">
-        <v>230</v>
+      <c r="B106" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="C106" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2022</v>
       </c>
-      <c r="B107" t="s">
-        <v>231</v>
+      <c r="B107" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="C107" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2022</v>
       </c>
-      <c r="B108" t="s">
-        <v>232</v>
+      <c r="B108" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="C108" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2022</v>
       </c>
-      <c r="B109" t="s">
-        <v>233</v>
+      <c r="B109" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="C109" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2022</v>
       </c>
-      <c r="B110" t="s">
-        <v>234</v>
+      <c r="B110" s="2" t="s">
+        <v>164</v>
       </c>
       <c r="C110" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2022</v>
       </c>
-      <c r="B111" t="s">
-        <v>235</v>
+      <c r="B111" s="2" t="s">
+        <v>165</v>
       </c>
       <c r="C111" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2022</v>
       </c>
-      <c r="B112" t="s">
-        <v>236</v>
+      <c r="B112" s="2" t="s">
+        <v>166</v>
       </c>
       <c r="C112" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2022</v>
       </c>
-      <c r="B113" t="s">
-        <v>237</v>
+      <c r="B113" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="C113" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2022</v>
       </c>
-      <c r="B114" t="s">
-        <v>238</v>
+      <c r="B114" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="C114" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2022</v>
       </c>
-      <c r="B115" t="s">
-        <v>239</v>
+      <c r="B115" s="2" t="s">
+        <v>169</v>
       </c>
       <c r="C115" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2022</v>
       </c>
-      <c r="B116" t="s">
-        <v>240</v>
+      <c r="B116" s="2" t="s">
+        <v>170</v>
       </c>
       <c r="C116" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2022</v>
       </c>
-      <c r="B117" t="s">
-        <v>241</v>
+      <c r="B117" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="C117" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2022</v>
       </c>
-      <c r="B118" t="s">
-        <v>242</v>
+      <c r="B118" s="2" t="s">
+        <v>172</v>
       </c>
       <c r="C118" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2022</v>
       </c>
-      <c r="B119" t="s">
-        <v>244</v>
+      <c r="B119" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="C119" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2022</v>
       </c>
-      <c r="B120" t="s">
-        <v>245</v>
+      <c r="B120" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="C120" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2022</v>
       </c>
-      <c r="B121" t="s">
-        <v>246</v>
+      <c r="B121" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="C121" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2023</v>
       </c>
-      <c r="B122" t="s">
-        <v>74</v>
+      <c r="B122" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="C122" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2023</v>
       </c>
-      <c r="B123" t="s">
-        <v>69</v>
+      <c r="B123" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="C123" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2023</v>
       </c>
-      <c r="B124" t="s">
-        <v>247</v>
+      <c r="B124" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="C124" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2023</v>
       </c>
-      <c r="B125" t="s">
-        <v>248</v>
+      <c r="B125" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="C125" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2023</v>
       </c>
-      <c r="B126" t="s">
-        <v>249</v>
+      <c r="B126" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="C126" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2023</v>
       </c>
-      <c r="B127" t="s">
-        <v>250</v>
+      <c r="B127" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="C127" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2023</v>
       </c>
-      <c r="B128" t="s">
-        <v>251</v>
+      <c r="B128" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="C128" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2023</v>
       </c>
-      <c r="B129" t="s">
-        <v>252</v>
+      <c r="B129" s="2" t="s">
+        <v>182</v>
       </c>
       <c r="C129" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2023</v>
       </c>
-      <c r="B130" t="s">
-        <v>253</v>
+      <c r="B130" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="C130" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2023</v>
       </c>
-      <c r="B131" t="s">
-        <v>254</v>
+      <c r="B131" s="2" t="s">
+        <v>184</v>
       </c>
       <c r="C131" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2023</v>
       </c>
-      <c r="B132" t="s">
-        <v>255</v>
+      <c r="B132" s="2" t="s">
+        <v>185</v>
       </c>
       <c r="C132" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2023</v>
       </c>
-      <c r="B133" t="s">
-        <v>256</v>
+      <c r="B133" s="2" t="s">
+        <v>186</v>
       </c>
       <c r="C133" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2023</v>
       </c>
-      <c r="B134" t="s">
-        <v>257</v>
+      <c r="B134" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="C134" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2023</v>
       </c>
-      <c r="B135" t="s">
-        <v>258</v>
+      <c r="B135" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="C135" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2023</v>
       </c>
-      <c r="B136" t="s">
-        <v>259</v>
+      <c r="B136" s="2" t="s">
+        <v>189</v>
       </c>
       <c r="C136" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2023</v>
       </c>
-      <c r="B137" t="s">
-        <v>260</v>
+      <c r="B137" s="2" t="s">
+        <v>190</v>
       </c>
       <c r="C137" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2023</v>
       </c>
-      <c r="B138" t="s">
-        <v>261</v>
+      <c r="B138" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="C138" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2023</v>
       </c>
-      <c r="B139" t="s">
-        <v>262</v>
+      <c r="B139" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="C139" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2023</v>
       </c>
-      <c r="B140" t="s">
-        <v>263</v>
+      <c r="B140" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="C140" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2023</v>
       </c>
-      <c r="B141" t="s">
-        <v>264</v>
+      <c r="B141" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="C141" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2023</v>
       </c>
-      <c r="B142" t="s">
-        <v>265</v>
+      <c r="B142" s="2" t="s">
+        <v>195</v>
       </c>
       <c r="C142" t="s">
-        <v>148</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -3917,7 +3708,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6471D813-4B53-4693-89A9-B1AB92C2992C}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>